<commit_message>
main01 and 02 sept
</commit_message>
<xml_diff>
--- a/12604997.xlsx
+++ b/12604997.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B27E255-0701-48A1-9905-0E76788D753A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EA02CD4-E354-467E-AA91-BBB2EDEE58A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -227,6 +227,9 @@
   </si>
   <si>
     <t>Feeling happy</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
 </sst>
 </file>
@@ -1282,48 +1285,96 @@
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="13"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="14"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="15" t="str">
+      <c r="A12" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B12" s="14">
+        <v>510</v>
+      </c>
+      <c r="C12" s="14">
+        <v>10</v>
+      </c>
+      <c r="D12" s="14">
+        <v>30</v>
+      </c>
+      <c r="E12" s="14">
+        <v>10</v>
+      </c>
+      <c r="F12" s="14">
+        <v>300</v>
+      </c>
+      <c r="G12" s="14">
+        <v>6</v>
+      </c>
+      <c r="H12" s="14">
+        <v>10</v>
+      </c>
+      <c r="I12" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="15" t="str">
+        <v>870</v>
+      </c>
+      <c r="J12" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K12" s="16"/>
-      <c r="L12" s="16"/>
-      <c r="M12" s="16"/>
-      <c r="N12" s="17"/>
+        <v>570</v>
+      </c>
+      <c r="K12" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L12" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M12" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A13" s="13"/>
-      <c r="B13" s="14"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="14"/>
-      <c r="I13" s="15" t="str">
+      <c r="A13" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B13" s="14">
+        <v>520</v>
+      </c>
+      <c r="C13" s="14">
+        <v>10</v>
+      </c>
+      <c r="D13" s="14">
+        <v>40</v>
+      </c>
+      <c r="E13" s="14">
+        <v>50</v>
+      </c>
+      <c r="F13" s="14">
+        <v>300</v>
+      </c>
+      <c r="G13" s="14">
+        <v>6</v>
+      </c>
+      <c r="H13" s="14">
+        <v>10</v>
+      </c>
+      <c r="I13" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="15" t="str">
+        <v>930</v>
+      </c>
+      <c r="J13" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K13" s="16"/>
-      <c r="L13" s="16"/>
-      <c r="M13" s="16"/>
-      <c r="N13" s="17"/>
+        <v>510</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>64</v>
+      </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>

</xml_diff>

<commit_message>
main10 and 11 sep
</commit_message>
<xml_diff>
--- a/12604997.xlsx
+++ b/12604997.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59497813-2218-4C96-8F1B-AADAC51D9926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC4229CC-BD10-4B46-AABA-13AAF666CDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="68">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -236,6 +236,9 @@
   </si>
   <si>
     <t>Na</t>
+  </si>
+  <si>
+    <t>Feeling better</t>
   </si>
 </sst>
 </file>
@@ -1698,55 +1701,103 @@
         <v>52</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="N20" s="17" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46275</v>
+      </c>
+      <c r="B21" s="14">
+        <v>550</v>
+      </c>
+      <c r="C21" s="14">
+        <v>45</v>
+      </c>
+      <c r="D21" s="14">
+        <v>90</v>
+      </c>
+      <c r="E21" s="14">
+        <v>45</v>
+      </c>
+      <c r="F21" s="14">
+        <v>150</v>
+      </c>
+      <c r="G21" s="14">
+        <v>3</v>
+      </c>
+      <c r="H21" s="14">
+        <v>35</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>915</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
+        <v>525</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46276</v>
+      </c>
+      <c r="B22" s="14">
+        <v>565</v>
+      </c>
+      <c r="C22" s="14">
+        <v>35</v>
+      </c>
+      <c r="D22" s="14">
+        <v>80</v>
+      </c>
+      <c r="E22" s="14">
+        <v>55</v>
+      </c>
+      <c r="F22" s="14">
+        <v>250</v>
+      </c>
+      <c r="G22" s="14">
+        <v>5</v>
+      </c>
+      <c r="H22" s="14">
+        <v>45</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="13"/>

</xml_diff>